<commit_message>
add J147 Method Heartrate binding to sat method ddba93dd23cb1d8115df3fe202503238d16b36e6
</commit_message>
<xml_diff>
--- a/ig/nr-add-sato2-profile/StructureDefinition-mesures-fr-observation-oxygen-sat.xlsx
+++ b/ig/nr-add-sato2-profile/StructureDefinition-mesures-fr-observation-oxygen-sat.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$110</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3839" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4260" uniqueCount="706">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-17T15:40:40+00:00</t>
+    <t>2023-11-23T10:07:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1786,16 +1786,46 @@
     <t>In some cases, method can impact results and is thus used for determining whether results can be compared or determining significance of results.</t>
   </si>
   <si>
-    <t>Methods for simple observations.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/observation-methods</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J147-MethodHeartrate-ENS/FHIR/JDV-J147-MethodHeartrate-ENS</t>
   </si>
   <si>
     <t>OBX-17</t>
   </si>
   <si>
     <t>methodCode</t>
+  </si>
+  <si>
+    <t>Observation.method.id</t>
+  </si>
+  <si>
+    <t>Observation.method.extension</t>
+  </si>
+  <si>
+    <t>Observation.method.coding</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.id</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.extension</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.system</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.version</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.code</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.display</t>
+  </si>
+  <si>
+    <t>Observation.method.coding.userSelected</t>
+  </si>
+  <si>
+    <t>Observation.method.text</t>
   </si>
   <si>
     <t>Observation.specimen</t>
@@ -2502,7 +2532,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP99"/>
+  <dimension ref="A1:AP110"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="56.234375" customWidth="true" bestFit="true"/>
@@ -2530,7 +2560,7 @@
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="98.61328125" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="85.6640625" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="93.578125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="42.03515625" customWidth="true" bestFit="true"/>
@@ -11675,13 +11705,11 @@
         <v>80</v>
       </c>
       <c r="X76" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="Y76" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="Y76" s="2"/>
+      <c r="Z76" t="s" s="2">
         <v>569</v>
-      </c>
-      <c r="Z76" t="s" s="2">
-        <v>570</v>
       </c>
       <c r="AA76" t="s" s="2">
         <v>80</v>
@@ -11720,10 +11748,10 @@
         <v>80</v>
       </c>
       <c r="AM76" t="s" s="2">
+        <v>570</v>
+      </c>
+      <c r="AN76" t="s" s="2">
         <v>571</v>
-      </c>
-      <c r="AN76" t="s" s="2">
-        <v>572</v>
       </c>
       <c r="AO76" t="s" s="2">
         <v>80</v>
@@ -11734,10 +11762,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -11760,17 +11788,15 @@
         <v>80</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>574</v>
+        <v>107</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>575</v>
+        <v>108</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>576</v>
-      </c>
-      <c r="N77" t="s" s="2">
-        <v>577</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N77" s="2"/>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
         <v>80</v>
@@ -11819,7 +11845,7 @@
         <v>80</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>573</v>
+        <v>110</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>78</v>
@@ -11828,47 +11854,47 @@
         <v>91</v>
       </c>
       <c r="AI77" t="s" s="2">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="AJ77" t="s" s="2">
-        <v>227</v>
+        <v>80</v>
       </c>
       <c r="AK77" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL77" t="s" s="2">
-        <v>578</v>
+        <v>80</v>
       </c>
       <c r="AM77" t="s" s="2">
-        <v>579</v>
+        <v>80</v>
       </c>
       <c r="AN77" t="s" s="2">
-        <v>580</v>
+        <v>111</v>
       </c>
       <c r="AO77" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP77" t="s" s="2">
-        <v>581</v>
+        <v>80</v>
       </c>
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="E78" s="2"/>
       <c r="F78" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G78" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H78" t="s" s="2">
         <v>80</v>
@@ -11880,16 +11906,16 @@
         <v>80</v>
       </c>
       <c r="K78" t="s" s="2">
-        <v>583</v>
+        <v>114</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>584</v>
+        <v>115</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>585</v>
+        <v>116</v>
       </c>
       <c r="N78" t="s" s="2">
-        <v>586</v>
+        <v>117</v>
       </c>
       <c r="O78" s="2"/>
       <c r="P78" t="s" s="2">
@@ -11927,57 +11953,57 @@
         <v>80</v>
       </c>
       <c r="AB78" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AC78" t="s" s="2">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="AD78" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE78" t="s" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>582</v>
+        <v>121</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH78" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI78" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ78" t="s" s="2">
-        <v>227</v>
+        <v>122</v>
       </c>
       <c r="AK78" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL78" t="s" s="2">
-        <v>587</v>
+        <v>80</v>
       </c>
       <c r="AM78" t="s" s="2">
-        <v>588</v>
+        <v>80</v>
       </c>
       <c r="AN78" t="s" s="2">
-        <v>589</v>
+        <v>105</v>
       </c>
       <c r="AO78" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP78" t="s" s="2">
-        <v>590</v>
+        <v>80</v>
       </c>
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>591</v>
+        <v>574</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>591</v>
+        <v>574</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11997,22 +12023,22 @@
         <v>80</v>
       </c>
       <c r="J79" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K79" t="s" s="2">
-        <v>592</v>
+        <v>147</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>593</v>
+        <v>300</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>594</v>
+        <v>301</v>
       </c>
       <c r="N79" t="s" s="2">
-        <v>595</v>
+        <v>302</v>
       </c>
       <c r="O79" t="s" s="2">
-        <v>596</v>
+        <v>303</v>
       </c>
       <c r="P79" t="s" s="2">
         <v>80</v>
@@ -12061,7 +12087,7 @@
         <v>80</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>591</v>
+        <v>304</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>78</v>
@@ -12073,7 +12099,7 @@
         <v>103</v>
       </c>
       <c r="AJ79" t="s" s="2">
-        <v>597</v>
+        <v>104</v>
       </c>
       <c r="AK79" t="s" s="2">
         <v>80</v>
@@ -12082,10 +12108,10 @@
         <v>80</v>
       </c>
       <c r="AM79" t="s" s="2">
-        <v>598</v>
+        <v>305</v>
       </c>
       <c r="AN79" t="s" s="2">
-        <v>599</v>
+        <v>306</v>
       </c>
       <c r="AO79" t="s" s="2">
         <v>80</v>
@@ -12096,10 +12122,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>600</v>
+        <v>575</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>600</v>
+        <v>575</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -12214,10 +12240,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>601</v>
+        <v>576</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>601</v>
+        <v>576</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -12334,45 +12360,45 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>602</v>
+        <v>577</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>602</v>
+        <v>577</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
-        <v>603</v>
+        <v>80</v>
       </c>
       <c r="E82" s="2"/>
       <c r="F82" t="s" s="2">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G82" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H82" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I82" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="J82" t="s" s="2">
         <v>92</v>
       </c>
       <c r="K82" t="s" s="2">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>604</v>
+        <v>313</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>605</v>
+        <v>314</v>
       </c>
       <c r="N82" t="s" s="2">
-        <v>117</v>
+        <v>315</v>
       </c>
       <c r="O82" t="s" s="2">
-        <v>209</v>
+        <v>316</v>
       </c>
       <c r="P82" t="s" s="2">
         <v>80</v>
@@ -12421,19 +12447,19 @@
         <v>80</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>606</v>
+        <v>318</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH82" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI82" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ82" t="s" s="2">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="AK82" t="s" s="2">
         <v>80</v>
@@ -12442,10 +12468,10 @@
         <v>80</v>
       </c>
       <c r="AM82" t="s" s="2">
-        <v>80</v>
+        <v>319</v>
       </c>
       <c r="AN82" t="s" s="2">
-        <v>105</v>
+        <v>320</v>
       </c>
       <c r="AO82" t="s" s="2">
         <v>80</v>
@@ -12456,10 +12482,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>607</v>
+        <v>578</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>607</v>
+        <v>578</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -12479,19 +12505,19 @@
         <v>80</v>
       </c>
       <c r="J83" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K83" t="s" s="2">
-        <v>608</v>
+        <v>107</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>609</v>
+        <v>323</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>610</v>
+        <v>324</v>
       </c>
       <c r="N83" t="s" s="2">
-        <v>611</v>
+        <v>325</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
@@ -12541,7 +12567,7 @@
         <v>80</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>607</v>
+        <v>326</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>78</v>
@@ -12550,10 +12576,10 @@
         <v>91</v>
       </c>
       <c r="AI83" t="s" s="2">
-        <v>612</v>
+        <v>103</v>
       </c>
       <c r="AJ83" t="s" s="2">
-        <v>613</v>
+        <v>104</v>
       </c>
       <c r="AK83" t="s" s="2">
         <v>80</v>
@@ -12562,10 +12588,10 @@
         <v>80</v>
       </c>
       <c r="AM83" t="s" s="2">
-        <v>614</v>
+        <v>327</v>
       </c>
       <c r="AN83" t="s" s="2">
-        <v>615</v>
+        <v>328</v>
       </c>
       <c r="AO83" t="s" s="2">
         <v>80</v>
@@ -12576,10 +12602,10 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>616</v>
+        <v>579</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>616</v>
+        <v>579</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -12587,7 +12613,7 @@
       </c>
       <c r="E84" s="2"/>
       <c r="F84" t="s" s="2">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G84" t="s" s="2">
         <v>91</v>
@@ -12599,21 +12625,23 @@
         <v>80</v>
       </c>
       <c r="J84" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K84" t="s" s="2">
-        <v>608</v>
+        <v>171</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>617</v>
+        <v>331</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>618</v>
+        <v>332</v>
       </c>
       <c r="N84" t="s" s="2">
-        <v>611</v>
-      </c>
-      <c r="O84" s="2"/>
+        <v>333</v>
+      </c>
+      <c r="O84" t="s" s="2">
+        <v>334</v>
+      </c>
       <c r="P84" t="s" s="2">
         <v>80</v>
       </c>
@@ -12661,7 +12689,7 @@
         <v>80</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>616</v>
+        <v>336</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>78</v>
@@ -12670,10 +12698,10 @@
         <v>91</v>
       </c>
       <c r="AI84" t="s" s="2">
-        <v>612</v>
+        <v>103</v>
       </c>
       <c r="AJ84" t="s" s="2">
-        <v>613</v>
+        <v>104</v>
       </c>
       <c r="AK84" t="s" s="2">
         <v>80</v>
@@ -12682,10 +12710,10 @@
         <v>80</v>
       </c>
       <c r="AM84" t="s" s="2">
-        <v>614</v>
+        <v>337</v>
       </c>
       <c r="AN84" t="s" s="2">
-        <v>619</v>
+        <v>338</v>
       </c>
       <c r="AO84" t="s" s="2">
         <v>80</v>
@@ -12696,10 +12724,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>620</v>
+        <v>580</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>620</v>
+        <v>580</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -12719,22 +12747,22 @@
         <v>80</v>
       </c>
       <c r="J85" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K85" t="s" s="2">
-        <v>281</v>
+        <v>107</v>
       </c>
       <c r="L85" t="s" s="2">
-        <v>621</v>
+        <v>341</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>622</v>
+        <v>342</v>
       </c>
       <c r="N85" t="s" s="2">
-        <v>623</v>
+        <v>333</v>
       </c>
       <c r="O85" t="s" s="2">
-        <v>624</v>
+        <v>343</v>
       </c>
       <c r="P85" t="s" s="2">
         <v>80</v>
@@ -12759,13 +12787,13 @@
         <v>80</v>
       </c>
       <c r="X85" t="s" s="2">
-        <v>175</v>
+        <v>80</v>
       </c>
       <c r="Y85" t="s" s="2">
-        <v>625</v>
+        <v>80</v>
       </c>
       <c r="Z85" t="s" s="2">
-        <v>626</v>
+        <v>80</v>
       </c>
       <c r="AA85" t="s" s="2">
         <v>80</v>
@@ -12783,7 +12811,7 @@
         <v>80</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>620</v>
+        <v>344</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>78</v>
@@ -12801,13 +12829,13 @@
         <v>80</v>
       </c>
       <c r="AL85" t="s" s="2">
-        <v>627</v>
+        <v>80</v>
       </c>
       <c r="AM85" t="s" s="2">
-        <v>628</v>
+        <v>345</v>
       </c>
       <c r="AN85" t="s" s="2">
-        <v>544</v>
+        <v>346</v>
       </c>
       <c r="AO85" t="s" s="2">
         <v>80</v>
@@ -12818,10 +12846,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>629</v>
+        <v>581</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>629</v>
+        <v>581</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -12832,7 +12860,7 @@
         <v>78</v>
       </c>
       <c r="G86" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H86" t="s" s="2">
         <v>80</v>
@@ -12841,22 +12869,22 @@
         <v>80</v>
       </c>
       <c r="J86" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>281</v>
+        <v>349</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>630</v>
+        <v>350</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>631</v>
+        <v>351</v>
       </c>
       <c r="N86" t="s" s="2">
-        <v>632</v>
+        <v>352</v>
       </c>
       <c r="O86" t="s" s="2">
-        <v>633</v>
+        <v>353</v>
       </c>
       <c r="P86" t="s" s="2">
         <v>80</v>
@@ -12881,13 +12909,13 @@
         <v>80</v>
       </c>
       <c r="X86" t="s" s="2">
-        <v>161</v>
+        <v>80</v>
       </c>
       <c r="Y86" t="s" s="2">
-        <v>634</v>
+        <v>80</v>
       </c>
       <c r="Z86" t="s" s="2">
-        <v>635</v>
+        <v>80</v>
       </c>
       <c r="AA86" t="s" s="2">
         <v>80</v>
@@ -12905,13 +12933,13 @@
         <v>80</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>629</v>
+        <v>354</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH86" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI86" t="s" s="2">
         <v>103</v>
@@ -12923,13 +12951,13 @@
         <v>80</v>
       </c>
       <c r="AL86" t="s" s="2">
-        <v>627</v>
+        <v>80</v>
       </c>
       <c r="AM86" t="s" s="2">
-        <v>628</v>
+        <v>355</v>
       </c>
       <c r="AN86" t="s" s="2">
-        <v>544</v>
+        <v>356</v>
       </c>
       <c r="AO86" t="s" s="2">
         <v>80</v>
@@ -12940,10 +12968,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>636</v>
+        <v>582</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>636</v>
+        <v>582</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -12963,22 +12991,22 @@
         <v>80</v>
       </c>
       <c r="J87" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K87" t="s" s="2">
-        <v>637</v>
+        <v>107</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>638</v>
+        <v>359</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>639</v>
+        <v>360</v>
       </c>
       <c r="N87" t="s" s="2">
-        <v>640</v>
+        <v>361</v>
       </c>
       <c r="O87" t="s" s="2">
-        <v>641</v>
+        <v>362</v>
       </c>
       <c r="P87" t="s" s="2">
         <v>80</v>
@@ -13027,7 +13055,7 @@
         <v>80</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>636</v>
+        <v>363</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>78</v>
@@ -13039,7 +13067,7 @@
         <v>103</v>
       </c>
       <c r="AJ87" t="s" s="2">
-        <v>642</v>
+        <v>104</v>
       </c>
       <c r="AK87" t="s" s="2">
         <v>80</v>
@@ -13048,10 +13076,10 @@
         <v>80</v>
       </c>
       <c r="AM87" t="s" s="2">
-        <v>643</v>
+        <v>364</v>
       </c>
       <c r="AN87" t="s" s="2">
-        <v>644</v>
+        <v>365</v>
       </c>
       <c r="AO87" t="s" s="2">
         <v>80</v>
@@ -13062,10 +13090,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>645</v>
+        <v>583</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>645</v>
+        <v>583</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -13088,16 +13116,16 @@
         <v>80</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>107</v>
+        <v>584</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>646</v>
+        <v>585</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>647</v>
+        <v>586</v>
       </c>
       <c r="N88" t="s" s="2">
-        <v>333</v>
+        <v>587</v>
       </c>
       <c r="O88" s="2"/>
       <c r="P88" t="s" s="2">
@@ -13147,7 +13175,7 @@
         <v>80</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>645</v>
+        <v>583</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>78</v>
@@ -13159,33 +13187,33 @@
         <v>103</v>
       </c>
       <c r="AJ88" t="s" s="2">
-        <v>104</v>
+        <v>227</v>
       </c>
       <c r="AK88" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL88" t="s" s="2">
-        <v>80</v>
+        <v>588</v>
       </c>
       <c r="AM88" t="s" s="2">
-        <v>614</v>
+        <v>589</v>
       </c>
       <c r="AN88" t="s" s="2">
-        <v>648</v>
+        <v>590</v>
       </c>
       <c r="AO88" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP88" t="s" s="2">
-        <v>80</v>
+        <v>591</v>
       </c>
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>649</v>
+        <v>592</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>649</v>
+        <v>592</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -13196,7 +13224,7 @@
         <v>78</v>
       </c>
       <c r="G89" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H89" t="s" s="2">
         <v>80</v>
@@ -13205,19 +13233,19 @@
         <v>80</v>
       </c>
       <c r="J89" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>650</v>
+        <v>593</v>
       </c>
       <c r="L89" t="s" s="2">
-        <v>651</v>
+        <v>594</v>
       </c>
       <c r="M89" t="s" s="2">
-        <v>652</v>
+        <v>595</v>
       </c>
       <c r="N89" t="s" s="2">
-        <v>653</v>
+        <v>596</v>
       </c>
       <c r="O89" s="2"/>
       <c r="P89" t="s" s="2">
@@ -13267,13 +13295,13 @@
         <v>80</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>649</v>
+        <v>592</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH89" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI89" t="s" s="2">
         <v>103</v>
@@ -13285,27 +13313,27 @@
         <v>80</v>
       </c>
       <c r="AL89" t="s" s="2">
-        <v>80</v>
+        <v>597</v>
       </c>
       <c r="AM89" t="s" s="2">
-        <v>654</v>
+        <v>598</v>
       </c>
       <c r="AN89" t="s" s="2">
-        <v>655</v>
+        <v>599</v>
       </c>
       <c r="AO89" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP89" t="s" s="2">
-        <v>80</v>
+        <v>600</v>
       </c>
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>656</v>
+        <v>601</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>656</v>
+        <v>601</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -13325,21 +13353,23 @@
         <v>80</v>
       </c>
       <c r="J90" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K90" t="s" s="2">
-        <v>657</v>
+        <v>602</v>
       </c>
       <c r="L90" t="s" s="2">
-        <v>658</v>
+        <v>603</v>
       </c>
       <c r="M90" t="s" s="2">
-        <v>659</v>
+        <v>604</v>
       </c>
       <c r="N90" t="s" s="2">
-        <v>660</v>
-      </c>
-      <c r="O90" s="2"/>
+        <v>605</v>
+      </c>
+      <c r="O90" t="s" s="2">
+        <v>606</v>
+      </c>
       <c r="P90" t="s" s="2">
         <v>80</v>
       </c>
@@ -13387,7 +13417,7 @@
         <v>80</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>656</v>
+        <v>601</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>78</v>
@@ -13399,7 +13429,7 @@
         <v>103</v>
       </c>
       <c r="AJ90" t="s" s="2">
-        <v>227</v>
+        <v>607</v>
       </c>
       <c r="AK90" t="s" s="2">
         <v>80</v>
@@ -13408,10 +13438,10 @@
         <v>80</v>
       </c>
       <c r="AM90" t="s" s="2">
-        <v>654</v>
+        <v>608</v>
       </c>
       <c r="AN90" t="s" s="2">
-        <v>661</v>
+        <v>609</v>
       </c>
       <c r="AO90" t="s" s="2">
         <v>80</v>
@@ -13422,10 +13452,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>662</v>
+        <v>610</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>662</v>
+        <v>610</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -13436,32 +13466,28 @@
         <v>78</v>
       </c>
       <c r="G91" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H91" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I91" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J91" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K91" t="s" s="2">
-        <v>592</v>
+        <v>107</v>
       </c>
       <c r="L91" t="s" s="2">
-        <v>663</v>
+        <v>108</v>
       </c>
       <c r="M91" t="s" s="2">
-        <v>663</v>
-      </c>
-      <c r="N91" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="O91" t="s" s="2">
-        <v>665</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N91" s="2"/>
+      <c r="O91" s="2"/>
       <c r="P91" t="s" s="2">
         <v>80</v>
       </c>
@@ -13509,19 +13535,19 @@
         <v>80</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>662</v>
+        <v>110</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH91" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI91" t="s" s="2">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="AJ91" t="s" s="2">
-        <v>666</v>
+        <v>80</v>
       </c>
       <c r="AK91" t="s" s="2">
         <v>80</v>
@@ -13530,10 +13556,10 @@
         <v>80</v>
       </c>
       <c r="AM91" t="s" s="2">
-        <v>667</v>
+        <v>80</v>
       </c>
       <c r="AN91" t="s" s="2">
-        <v>668</v>
+        <v>111</v>
       </c>
       <c r="AO91" t="s" s="2">
         <v>80</v>
@@ -13544,21 +13570,21 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>669</v>
+        <v>611</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>669</v>
+        <v>611</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="E92" s="2"/>
       <c r="F92" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G92" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H92" t="s" s="2">
         <v>80</v>
@@ -13570,15 +13596,17 @@
         <v>80</v>
       </c>
       <c r="K92" t="s" s="2">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="M92" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="N92" s="2"/>
+        <v>116</v>
+      </c>
+      <c r="N92" t="s" s="2">
+        <v>117</v>
+      </c>
       <c r="O92" s="2"/>
       <c r="P92" t="s" s="2">
         <v>80</v>
@@ -13615,31 +13643,31 @@
         <v>80</v>
       </c>
       <c r="AB92" t="s" s="2">
-        <v>80</v>
+        <v>118</v>
       </c>
       <c r="AC92" t="s" s="2">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="AD92" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE92" t="s" s="2">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="AF92" t="s" s="2">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="AG92" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH92" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI92" t="s" s="2">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="AJ92" t="s" s="2">
-        <v>80</v>
+        <v>122</v>
       </c>
       <c r="AK92" t="s" s="2">
         <v>80</v>
@@ -13651,7 +13679,7 @@
         <v>80</v>
       </c>
       <c r="AN92" t="s" s="2">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="AO92" t="s" s="2">
         <v>80</v>
@@ -13662,14 +13690,14 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>670</v>
+        <v>612</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>670</v>
+        <v>612</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
-        <v>113</v>
+        <v>613</v>
       </c>
       <c r="E93" s="2"/>
       <c r="F93" t="s" s="2">
@@ -13682,24 +13710,26 @@
         <v>80</v>
       </c>
       <c r="I93" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="J93" t="s" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K93" t="s" s="2">
         <v>114</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>115</v>
+        <v>614</v>
       </c>
       <c r="M93" t="s" s="2">
-        <v>116</v>
+        <v>615</v>
       </c>
       <c r="N93" t="s" s="2">
         <v>117</v>
       </c>
-      <c r="O93" s="2"/>
+      <c r="O93" t="s" s="2">
+        <v>209</v>
+      </c>
       <c r="P93" t="s" s="2">
         <v>80</v>
       </c>
@@ -13735,19 +13765,19 @@
         <v>80</v>
       </c>
       <c r="AB93" t="s" s="2">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="AC93" t="s" s="2">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="AD93" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE93" t="s" s="2">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="AF93" t="s" s="2">
-        <v>121</v>
+        <v>616</v>
       </c>
       <c r="AG93" t="s" s="2">
         <v>78</v>
@@ -13782,46 +13812,44 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>671</v>
+        <v>617</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>671</v>
+        <v>617</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
-        <v>603</v>
+        <v>80</v>
       </c>
       <c r="E94" s="2"/>
       <c r="F94" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G94" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H94" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I94" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="J94" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K94" t="s" s="2">
-        <v>114</v>
+        <v>618</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>604</v>
+        <v>619</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>605</v>
+        <v>620</v>
       </c>
       <c r="N94" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="O94" t="s" s="2">
-        <v>209</v>
-      </c>
+        <v>621</v>
+      </c>
+      <c r="O94" s="2"/>
       <c r="P94" t="s" s="2">
         <v>80</v>
       </c>
@@ -13869,19 +13897,19 @@
         <v>80</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>606</v>
+        <v>617</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH94" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI94" t="s" s="2">
-        <v>103</v>
+        <v>622</v>
       </c>
       <c r="AJ94" t="s" s="2">
-        <v>122</v>
+        <v>623</v>
       </c>
       <c r="AK94" t="s" s="2">
         <v>80</v>
@@ -13890,10 +13918,10 @@
         <v>80</v>
       </c>
       <c r="AM94" t="s" s="2">
-        <v>80</v>
+        <v>624</v>
       </c>
       <c r="AN94" t="s" s="2">
-        <v>105</v>
+        <v>625</v>
       </c>
       <c r="AO94" t="s" s="2">
         <v>80</v>
@@ -13904,10 +13932,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>672</v>
+        <v>626</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>672</v>
+        <v>626</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -13915,35 +13943,33 @@
       </c>
       <c r="E95" s="2"/>
       <c r="F95" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G95" t="s" s="2">
         <v>91</v>
       </c>
       <c r="H95" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J95" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>281</v>
+        <v>618</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>673</v>
+        <v>627</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>674</v>
+        <v>628</v>
       </c>
       <c r="N95" t="s" s="2">
-        <v>675</v>
-      </c>
-      <c r="O95" t="s" s="2">
-        <v>676</v>
-      </c>
+        <v>621</v>
+      </c>
+      <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
         <v>80</v>
       </c>
@@ -13967,13 +13993,13 @@
         <v>80</v>
       </c>
       <c r="X95" t="s" s="2">
-        <v>151</v>
+        <v>80</v>
       </c>
       <c r="Y95" t="s" s="2">
-        <v>372</v>
+        <v>80</v>
       </c>
       <c r="Z95" t="s" s="2">
-        <v>373</v>
+        <v>80</v>
       </c>
       <c r="AA95" t="s" s="2">
         <v>80</v>
@@ -13991,34 +14017,34 @@
         <v>80</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>672</v>
+        <v>626</v>
       </c>
       <c r="AG95" t="s" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="AH95" t="s" s="2">
         <v>91</v>
       </c>
       <c r="AI95" t="s" s="2">
-        <v>103</v>
+        <v>622</v>
       </c>
       <c r="AJ95" t="s" s="2">
-        <v>104</v>
+        <v>623</v>
       </c>
       <c r="AK95" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL95" t="s" s="2">
-        <v>677</v>
+        <v>80</v>
       </c>
       <c r="AM95" t="s" s="2">
-        <v>376</v>
+        <v>624</v>
       </c>
       <c r="AN95" t="s" s="2">
-        <v>377</v>
+        <v>629</v>
       </c>
       <c r="AO95" t="s" s="2">
-        <v>378</v>
+        <v>80</v>
       </c>
       <c r="AP95" t="s" s="2">
         <v>80</v>
@@ -14026,10 +14052,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>678</v>
+        <v>630</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>678</v>
+        <v>630</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -14043,28 +14069,28 @@
         <v>91</v>
       </c>
       <c r="H96" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I96" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J96" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="K96" t="s" s="2">
-        <v>460</v>
+        <v>281</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>679</v>
+        <v>631</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>680</v>
+        <v>632</v>
       </c>
       <c r="N96" t="s" s="2">
-        <v>681</v>
+        <v>633</v>
       </c>
       <c r="O96" t="s" s="2">
-        <v>463</v>
+        <v>634</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>80</v>
@@ -14089,13 +14115,13 @@
         <v>80</v>
       </c>
       <c r="X96" t="s" s="2">
-        <v>272</v>
+        <v>175</v>
       </c>
       <c r="Y96" t="s" s="2">
-        <v>682</v>
+        <v>635</v>
       </c>
       <c r="Z96" t="s" s="2">
-        <v>683</v>
+        <v>636</v>
       </c>
       <c r="AA96" t="s" s="2">
         <v>80</v>
@@ -14113,7 +14139,7 @@
         <v>80</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>678</v>
+        <v>630</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>78</v>
@@ -14122,7 +14148,7 @@
         <v>91</v>
       </c>
       <c r="AI96" t="s" s="2">
-        <v>684</v>
+        <v>103</v>
       </c>
       <c r="AJ96" t="s" s="2">
         <v>104</v>
@@ -14131,27 +14157,27 @@
         <v>80</v>
       </c>
       <c r="AL96" t="s" s="2">
-        <v>685</v>
+        <v>637</v>
       </c>
       <c r="AM96" t="s" s="2">
-        <v>468</v>
+        <v>638</v>
       </c>
       <c r="AN96" t="s" s="2">
-        <v>469</v>
+        <v>544</v>
       </c>
       <c r="AO96" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP96" t="s" s="2">
-        <v>470</v>
+        <v>80</v>
       </c>
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>686</v>
+        <v>639</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>686</v>
+        <v>639</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -14162,10 +14188,10 @@
         <v>78</v>
       </c>
       <c r="G97" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H97" t="s" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="I97" t="s" s="2">
         <v>80</v>
@@ -14177,16 +14203,16 @@
         <v>281</v>
       </c>
       <c r="L97" t="s" s="2">
-        <v>687</v>
+        <v>640</v>
       </c>
       <c r="M97" t="s" s="2">
-        <v>688</v>
+        <v>641</v>
       </c>
       <c r="N97" t="s" s="2">
-        <v>689</v>
+        <v>642</v>
       </c>
       <c r="O97" t="s" s="2">
-        <v>529</v>
+        <v>643</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>80</v>
@@ -14211,13 +14237,13 @@
         <v>80</v>
       </c>
       <c r="X97" t="s" s="2">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="Y97" t="s" s="2">
-        <v>530</v>
+        <v>644</v>
       </c>
       <c r="Z97" t="s" s="2">
-        <v>531</v>
+        <v>645</v>
       </c>
       <c r="AA97" t="s" s="2">
         <v>80</v>
@@ -14235,16 +14261,16 @@
         <v>80</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>686</v>
+        <v>639</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH97" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AI97" t="s" s="2">
-        <v>690</v>
+        <v>103</v>
       </c>
       <c r="AJ97" t="s" s="2">
         <v>104</v>
@@ -14253,13 +14279,13 @@
         <v>80</v>
       </c>
       <c r="AL97" t="s" s="2">
-        <v>80</v>
+        <v>637</v>
       </c>
       <c r="AM97" t="s" s="2">
-        <v>105</v>
+        <v>638</v>
       </c>
       <c r="AN97" t="s" s="2">
-        <v>533</v>
+        <v>544</v>
       </c>
       <c r="AO97" t="s" s="2">
         <v>80</v>
@@ -14270,21 +14296,21 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>691</v>
+        <v>646</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>691</v>
+        <v>646</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
-        <v>535</v>
+        <v>80</v>
       </c>
       <c r="E98" s="2"/>
       <c r="F98" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G98" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H98" t="s" s="2">
         <v>80</v>
@@ -14296,19 +14322,19 @@
         <v>80</v>
       </c>
       <c r="K98" t="s" s="2">
-        <v>281</v>
+        <v>647</v>
       </c>
       <c r="L98" t="s" s="2">
-        <v>536</v>
+        <v>648</v>
       </c>
       <c r="M98" t="s" s="2">
-        <v>537</v>
+        <v>649</v>
       </c>
       <c r="N98" t="s" s="2">
-        <v>538</v>
+        <v>650</v>
       </c>
       <c r="O98" t="s" s="2">
-        <v>539</v>
+        <v>651</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>80</v>
@@ -14333,13 +14359,13 @@
         <v>80</v>
       </c>
       <c r="X98" t="s" s="2">
-        <v>151</v>
+        <v>80</v>
       </c>
       <c r="Y98" t="s" s="2">
-        <v>540</v>
+        <v>80</v>
       </c>
       <c r="Z98" t="s" s="2">
-        <v>692</v>
+        <v>80</v>
       </c>
       <c r="AA98" t="s" s="2">
         <v>80</v>
@@ -14357,45 +14383,45 @@
         <v>80</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>691</v>
+        <v>646</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH98" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AI98" t="s" s="2">
         <v>103</v>
       </c>
       <c r="AJ98" t="s" s="2">
-        <v>104</v>
+        <v>652</v>
       </c>
       <c r="AK98" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL98" t="s" s="2">
-        <v>542</v>
+        <v>80</v>
       </c>
       <c r="AM98" t="s" s="2">
-        <v>543</v>
+        <v>653</v>
       </c>
       <c r="AN98" t="s" s="2">
-        <v>544</v>
+        <v>654</v>
       </c>
       <c r="AO98" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP98" t="s" s="2">
-        <v>545</v>
+        <v>80</v>
       </c>
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>693</v>
+        <v>655</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>693</v>
+        <v>655</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -14406,7 +14432,7 @@
         <v>78</v>
       </c>
       <c r="G99" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H99" t="s" s="2">
         <v>80</v>
@@ -14418,20 +14444,18 @@
         <v>80</v>
       </c>
       <c r="K99" t="s" s="2">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>694</v>
+        <v>656</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>695</v>
+        <v>657</v>
       </c>
       <c r="N99" t="s" s="2">
-        <v>595</v>
-      </c>
-      <c r="O99" t="s" s="2">
-        <v>596</v>
-      </c>
+        <v>333</v>
+      </c>
+      <c r="O99" s="2"/>
       <c r="P99" t="s" s="2">
         <v>80</v>
       </c>
@@ -14479,41 +14503,1373 @@
         <v>80</v>
       </c>
       <c r="AF99" t="s" s="2">
+        <v>655</v>
+      </c>
+      <c r="AG99" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH99" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI99" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ99" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK99" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL99" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM99" t="s" s="2">
+        <v>624</v>
+      </c>
+      <c r="AN99" t="s" s="2">
+        <v>658</v>
+      </c>
+      <c r="AO99" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP99" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="100" hidden="true">
+      <c r="A100" t="s" s="2">
+        <v>659</v>
+      </c>
+      <c r="B100" t="s" s="2">
+        <v>659</v>
+      </c>
+      <c r="C100" s="2"/>
+      <c r="D100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E100" s="2"/>
+      <c r="F100" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G100" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J100" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K100" t="s" s="2">
+        <v>660</v>
+      </c>
+      <c r="L100" t="s" s="2">
+        <v>661</v>
+      </c>
+      <c r="M100" t="s" s="2">
+        <v>662</v>
+      </c>
+      <c r="N100" t="s" s="2">
+        <v>663</v>
+      </c>
+      <c r="O100" s="2"/>
+      <c r="P100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q100" s="2"/>
+      <c r="R100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF100" t="s" s="2">
+        <v>659</v>
+      </c>
+      <c r="AG100" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH100" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI100" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ100" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="AK100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM100" t="s" s="2">
+        <v>664</v>
+      </c>
+      <c r="AN100" t="s" s="2">
+        <v>665</v>
+      </c>
+      <c r="AO100" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP100" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="101" hidden="true">
+      <c r="A101" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="B101" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="C101" s="2"/>
+      <c r="D101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E101" s="2"/>
+      <c r="F101" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G101" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J101" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K101" t="s" s="2">
+        <v>667</v>
+      </c>
+      <c r="L101" t="s" s="2">
+        <v>668</v>
+      </c>
+      <c r="M101" t="s" s="2">
+        <v>669</v>
+      </c>
+      <c r="N101" t="s" s="2">
+        <v>670</v>
+      </c>
+      <c r="O101" s="2"/>
+      <c r="P101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q101" s="2"/>
+      <c r="R101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF101" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="AG101" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH101" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI101" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ101" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="AK101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM101" t="s" s="2">
+        <v>664</v>
+      </c>
+      <c r="AN101" t="s" s="2">
+        <v>671</v>
+      </c>
+      <c r="AO101" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP101" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="102" hidden="true">
+      <c r="A102" t="s" s="2">
+        <v>672</v>
+      </c>
+      <c r="B102" t="s" s="2">
+        <v>672</v>
+      </c>
+      <c r="C102" s="2"/>
+      <c r="D102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E102" s="2"/>
+      <c r="F102" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G102" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H102" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J102" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K102" t="s" s="2">
+        <v>602</v>
+      </c>
+      <c r="L102" t="s" s="2">
+        <v>673</v>
+      </c>
+      <c r="M102" t="s" s="2">
+        <v>673</v>
+      </c>
+      <c r="N102" t="s" s="2">
+        <v>674</v>
+      </c>
+      <c r="O102" t="s" s="2">
+        <v>675</v>
+      </c>
+      <c r="P102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q102" s="2"/>
+      <c r="R102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF102" t="s" s="2">
+        <v>672</v>
+      </c>
+      <c r="AG102" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH102" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI102" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ102" t="s" s="2">
+        <v>676</v>
+      </c>
+      <c r="AK102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM102" t="s" s="2">
+        <v>677</v>
+      </c>
+      <c r="AN102" t="s" s="2">
+        <v>678</v>
+      </c>
+      <c r="AO102" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP102" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="103" hidden="true">
+      <c r="A103" t="s" s="2">
+        <v>679</v>
+      </c>
+      <c r="B103" t="s" s="2">
+        <v>679</v>
+      </c>
+      <c r="C103" s="2"/>
+      <c r="D103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E103" s="2"/>
+      <c r="F103" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G103" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K103" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="L103" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="M103" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="N103" s="2"/>
+      <c r="O103" s="2"/>
+      <c r="P103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q103" s="2"/>
+      <c r="R103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF103" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="AG103" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH103" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AK103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN103" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="AO103" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP103" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="104" hidden="true">
+      <c r="A104" t="s" s="2">
+        <v>680</v>
+      </c>
+      <c r="B104" t="s" s="2">
+        <v>680</v>
+      </c>
+      <c r="C104" s="2"/>
+      <c r="D104" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="E104" s="2"/>
+      <c r="F104" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G104" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K104" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="L104" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="M104" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="N104" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="O104" s="2"/>
+      <c r="P104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q104" s="2"/>
+      <c r="R104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB104" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="AC104" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AD104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE104" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="AF104" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="AG104" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH104" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI104" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ104" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN104" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AO104" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP104" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="105" hidden="true">
+      <c r="A105" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="B105" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="C105" s="2"/>
+      <c r="D105" t="s" s="2">
+        <v>613</v>
+      </c>
+      <c r="E105" s="2"/>
+      <c r="F105" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G105" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I105" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="J105" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K105" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="L105" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="M105" t="s" s="2">
+        <v>615</v>
+      </c>
+      <c r="N105" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="O105" t="s" s="2">
+        <v>209</v>
+      </c>
+      <c r="P105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q105" s="2"/>
+      <c r="R105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF105" t="s" s="2">
+        <v>616</v>
+      </c>
+      <c r="AG105" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH105" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI105" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ105" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="AK105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN105" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AO105" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP105" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="106" hidden="true">
+      <c r="A106" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="B106" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="C106" s="2"/>
+      <c r="D106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E106" s="2"/>
+      <c r="F106" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="G106" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H106" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J106" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K106" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="L106" t="s" s="2">
+        <v>683</v>
+      </c>
+      <c r="M106" t="s" s="2">
+        <v>684</v>
+      </c>
+      <c r="N106" t="s" s="2">
+        <v>685</v>
+      </c>
+      <c r="O106" t="s" s="2">
+        <v>686</v>
+      </c>
+      <c r="P106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q106" s="2"/>
+      <c r="R106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X106" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="Y106" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="Z106" t="s" s="2">
+        <v>373</v>
+      </c>
+      <c r="AA106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF106" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="AG106" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AH106" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI106" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ106" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK106" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL106" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="AM106" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="AN106" t="s" s="2">
+        <v>377</v>
+      </c>
+      <c r="AO106" t="s" s="2">
+        <v>378</v>
+      </c>
+      <c r="AP106" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="107" hidden="true">
+      <c r="A107" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="B107" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="C107" s="2"/>
+      <c r="D107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E107" s="2"/>
+      <c r="F107" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G107" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H107" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J107" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="K107" t="s" s="2">
+        <v>460</v>
+      </c>
+      <c r="L107" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="M107" t="s" s="2">
+        <v>690</v>
+      </c>
+      <c r="N107" t="s" s="2">
+        <v>691</v>
+      </c>
+      <c r="O107" t="s" s="2">
+        <v>463</v>
+      </c>
+      <c r="P107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q107" s="2"/>
+      <c r="R107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X107" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="Y107" t="s" s="2">
+        <v>692</v>
+      </c>
+      <c r="Z107" t="s" s="2">
         <v>693</v>
       </c>
-      <c r="AG99" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH99" t="s" s="2">
+      <c r="AA107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF107" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="AG107" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH107" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI107" t="s" s="2">
+        <v>694</v>
+      </c>
+      <c r="AJ107" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL107" t="s" s="2">
+        <v>695</v>
+      </c>
+      <c r="AM107" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="AN107" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="AO107" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP107" t="s" s="2">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="108" hidden="true">
+      <c r="A108" t="s" s="2">
+        <v>696</v>
+      </c>
+      <c r="B108" t="s" s="2">
+        <v>696</v>
+      </c>
+      <c r="C108" s="2"/>
+      <c r="D108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E108" s="2"/>
+      <c r="F108" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G108" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H108" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K108" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="L108" t="s" s="2">
+        <v>697</v>
+      </c>
+      <c r="M108" t="s" s="2">
+        <v>698</v>
+      </c>
+      <c r="N108" t="s" s="2">
+        <v>699</v>
+      </c>
+      <c r="O108" t="s" s="2">
+        <v>529</v>
+      </c>
+      <c r="P108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q108" s="2"/>
+      <c r="R108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X108" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="Y108" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="Z108" t="s" s="2">
+        <v>531</v>
+      </c>
+      <c r="AA108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF108" t="s" s="2">
+        <v>696</v>
+      </c>
+      <c r="AG108" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH108" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI108" t="s" s="2">
+        <v>700</v>
+      </c>
+      <c r="AJ108" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM108" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AN108" t="s" s="2">
+        <v>533</v>
+      </c>
+      <c r="AO108" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP108" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="109" hidden="true">
+      <c r="A109" t="s" s="2">
+        <v>701</v>
+      </c>
+      <c r="B109" t="s" s="2">
+        <v>701</v>
+      </c>
+      <c r="C109" s="2"/>
+      <c r="D109" t="s" s="2">
+        <v>535</v>
+      </c>
+      <c r="E109" s="2"/>
+      <c r="F109" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G109" t="s" s="2">
         <v>79</v>
       </c>
-      <c r="AI99" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ99" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AK99" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AL99" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AM99" t="s" s="2">
-        <v>598</v>
-      </c>
-      <c r="AN99" t="s" s="2">
-        <v>599</v>
-      </c>
-      <c r="AO99" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP99" t="s" s="2">
+      <c r="H109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K109" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="L109" t="s" s="2">
+        <v>536</v>
+      </c>
+      <c r="M109" t="s" s="2">
+        <v>537</v>
+      </c>
+      <c r="N109" t="s" s="2">
+        <v>538</v>
+      </c>
+      <c r="O109" t="s" s="2">
+        <v>539</v>
+      </c>
+      <c r="P109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q109" s="2"/>
+      <c r="R109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X109" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="Y109" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="Z109" t="s" s="2">
+        <v>702</v>
+      </c>
+      <c r="AA109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF109" t="s" s="2">
+        <v>701</v>
+      </c>
+      <c r="AG109" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH109" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI109" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AJ109" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AK109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL109" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="AM109" t="s" s="2">
+        <v>543</v>
+      </c>
+      <c r="AN109" t="s" s="2">
+        <v>544</v>
+      </c>
+      <c r="AO109" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP109" t="s" s="2">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="110" hidden="true">
+      <c r="A110" t="s" s="2">
+        <v>703</v>
+      </c>
+      <c r="B110" t="s" s="2">
+        <v>703</v>
+      </c>
+      <c r="C110" s="2"/>
+      <c r="D110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E110" s="2"/>
+      <c r="F110" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G110" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K110" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="L110" t="s" s="2">
+        <v>704</v>
+      </c>
+      <c r="M110" t="s" s="2">
+        <v>705</v>
+      </c>
+      <c r="N110" t="s" s="2">
+        <v>605</v>
+      </c>
+      <c r="O110" t="s" s="2">
+        <v>606</v>
+      </c>
+      <c r="P110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q110" s="2"/>
+      <c r="R110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF110" t="s" s="2">
+        <v>703</v>
+      </c>
+      <c r="AG110" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH110" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AK110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM110" t="s" s="2">
+        <v>608</v>
+      </c>
+      <c r="AN110" t="s" s="2">
+        <v>609</v>
+      </c>
+      <c r="AO110" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP110" t="s" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP99">
+  <autoFilter ref="A1:AP110">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -14523,7 +15879,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI98">
+  <conditionalFormatting sqref="A2:AI109">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>